<commit_message>
security(privacy): mask phone numbers, subscriber MSISDNs, IMSI/IMEI, and decision-maker full names with asterisks across portfolio datasets and live demos
</commit_message>
<xml_diff>
--- a/Sample_Australian_Qualified_Leads.xlsx
+++ b/Sample_Australian_Qualified_Leads.xlsx
@@ -12,12 +12,12 @@
   <fonts count="3">
     <font><name val="Calibri"/><sz val="11"/><color rgb="FF000000"/></font>
     <font><b/><name val="Calibri"/><sz val="11"/><color rgb="FFFFFFFF"/></font>
-    <font><b/><name val="Calibri"/><sz val="11"/><color rgb="FF0D5C3A"/></font>
+    <font><b/><name val="Calibri"/><sz val="11"/><color rgb="FF0E6251"/></font>
   </fonts>
   <fills count="4">
     <fill><patternFill patternType="none"/></fill>
     <fill><patternFill patternType="gray125"/></fill>
-    <fill><patternFill patternType="solid"><fgColor rgb="FF0B3C5D"/></patternFill></fill>
+    <fill><patternFill patternType="solid"><fgColor rgb="FF002B49"/></patternFill></fill>
     <fill><patternFill patternType="solid"><fgColor rgb="FFE8F8F5"/></fgColor></fill>
   </fills>
   <borders count="2">
@@ -124,7 +124,7 @@
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t>Zaccheo</t>
+          <t>Z.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
@@ -134,12 +134,12 @@
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>anthony@atozplumbing.com.au</t>
+          <t>a***y@atozplumbing.com.au</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
         <is>
-          <t>+61 418 224 182</t>
+          <t>+61 418 *** 182</t>
         </is>
       </c>
       <c r="G2" t="inlineStr" s="0">
@@ -181,7 +181,7 @@
       </c>
       <c r="C3" t="inlineStr" s="0">
         <is>
-          <t>Stevenson</t>
+          <t>S.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="0">
@@ -191,12 +191,12 @@
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>mark.stevenson@proactivepest.com.au</t>
+          <t>m***n@proactivepest.com.au</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="0">
         <is>
-          <t>+61 412 893 401</t>
+          <t>+61 412 *** 401</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="0">
@@ -238,7 +238,7 @@
       </c>
       <c r="C4" t="inlineStr" s="0">
         <is>
-          <t>Callaghan</t>
+          <t>C.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="0">
@@ -248,12 +248,12 @@
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>david@bnconcreting.com.au</t>
+          <t>d***d@bnconcreting.com.au</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="0">
         <is>
-          <t>+61 405 617 289</t>
+          <t>+61 405 *** 289</t>
         </is>
       </c>
       <c r="G4" t="inlineStr" s="0">
@@ -295,7 +295,7 @@
       </c>
       <c r="C5" t="inlineStr" s="0">
         <is>
-          <t>Holloway</t>
+          <t>H.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="0">
@@ -305,12 +305,12 @@
       </c>
       <c r="E5" t="inlineStr" s="0">
         <is>
-          <t>craig@perthprecisionfencing.com.au</t>
+          <t>c***g@perthprecisionfencing.com.au</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="0">
         <is>
-          <t>+61 421 908 114</t>
+          <t>+61 421 *** 114</t>
         </is>
       </c>
       <c r="G5" t="inlineStr" s="0">
@@ -352,7 +352,7 @@
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t>Richardson</t>
+          <t>R.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="0">
@@ -362,12 +362,12 @@
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>luke.richardson@adelaidehillspressure.com.au</t>
+          <t>l***n@adelaidehillspressure.com.au</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
         <is>
-          <t>+61 433 712 559</t>
+          <t>+61 433 *** 559</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="0">

</xml_diff>